<commit_message>
Add gross margin comparison and dicing/packaging backend cost sections
New sections added to the spreadsheet:

GROSS MARGIN COMPARISON:
- TSMC corporate: 59.9% GM (FY2025), 62.3% Q4 2025
- Arizona fab: ~8% estimated GM (5nm) vs ~50-60% for Taiwan fabs
- Arizona first profitable year: NT$161.4B ($5.15B) in 2025
- Wafer price premium: 5-20% for AZ-made chips
- Margin dilution: 1-2% impact on corporate GM (2025)
- Key differentiator: cultural efficiencies priced explicitly in US

DICING, PACKAGING & BACKEND COSTS:
- AZ wafers currently flown back to Taiwan for all backend
- Air freight: ~$50-150/wafer added cost
- Dicing: ~$30-80/wafer (blade/laser)
- Packaging breakdown: FC-BGA $8, InFO $15, CoWoS-S $70,
  CoWoS-L $84-98, SoIC $120 per unit
- Full backend for AI chips: ~$750-1,100/chip
- Backend is 10-20% of std chip cost, 20-30% for AI/HPC
- OSAT prices rising 8-20% (2025-2026)

Sources expanded from 42 to 64 cited references.

Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/TSMC_Phoenix_vs_Taiwan_Fab_Costs.xlsx
+++ b/TSMC_Phoenix_vs_Taiwan_Fab_Costs.xlsx
@@ -535,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1471,7 +1471,7 @@
     <row r="38" ht="25" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>OVERALL WAFER PROCESSING COST</t>
+          <t>DICING, PACKAGING &amp; BACKEND COSTS (AZ-MADE CHIPS)</t>
         </is>
       </c>
       <c r="B38" s="5" t="n"/>
@@ -1483,75 +1483,773 @@
     <row r="39" ht="65" customHeight="1">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>Total Wafer Processing Cost (300mm, N4/N3)</t>
+          <t>Backend Process Flow (AZ chips)</t>
         </is>
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>~$17,000–$22,000/wafer</t>
+          <t>Wafers air-freighted to Taiwan for dicing, test &amp; packaging</t>
         </is>
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>~$15,500–$20,000/wafer</t>
-        </is>
-      </c>
-      <c r="D39" s="13" t="inlineStr">
-        <is>
-          <t>AZ ~10% higher overall</t>
+          <t>Dicing, test &amp; packaging done on-site or nearby OSAT (ASE/SPIL)</t>
+        </is>
+      </c>
+      <c r="D39" s="12" t="inlineStr">
+        <is>
+          <t>AZ adds logistics loop</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr">
         <is>
-          <t>Per TechInsights Strategic Cost &amp; Price Model (Scotten Jones). Equipment dominance (~67%+ of cost) equalizes locations. Total difference is &lt;10%.</t>
+          <t>AZ wafers currently fly back to Taiwan via Eva Air for all backend processing (dicing, wafer probe, packaging, final test), then ship to end customers or assembly sites. This adds ~2–4 weeks transit time.</t>
         </is>
       </c>
       <c r="F39" s="8" t="inlineStr">
         <is>
-          <t>TechInsights Mar 2025 (Chip Insider, G. Dan Hutcheson); Silicon Analysts 2026; SemiWiki</t>
+          <t>SemiWiki (AZ chips flown to TW); TechPowerUp Feb 2025; inkl.com Mar 2025</t>
         </is>
       </c>
     </row>
     <row r="40" ht="65" customHeight="1">
       <c r="A40" s="6" t="inlineStr">
         <is>
+          <t>Air Freight Cost (AZ→TW round trip)</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>Estimated ~$50–$150/wafer (specialized handling)</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>N/A (no shipping needed)</t>
+        </is>
+      </c>
+      <c r="D40" s="10" t="inlineStr">
+        <is>
+          <t>Added AZ cost</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>300mm wafers require specialized FOUPs, temperature/vibration control, and insurance. Air freight Taiwan↔USA is 1–5 days. Cost is modest per-wafer but adds up at volume; exact rates are negotiated privately.</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>Wafer World (wafer shipping guide); FreightAmigo (TW→US routes); industry estimates</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="65" customHeight="1">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>Wafer Dicing</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>Done in Taiwan (same cost as TW-made wafers + freight)</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>~$30–$80/wafer (blade or laser dicing, 300mm)</t>
+        </is>
+      </c>
+      <c r="D41" s="12" t="inlineStr">
+        <is>
+          <t>AZ adds freight overhead</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Dicing cost itself is location-independent since performed in Taiwan for both. Laser dicing (&gt;42% market share) used for advanced nodes with thin wafers and 3D stacking. Global dicing services market: $614M (2024).</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>Astute Analytica (dicing market); Han's Laser (300mm dicing methods); industry estimates</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="65" customHeight="1">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>Wafer Probe / Wafer-Level Test</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>Done in Taiwan (same cost as TW-made wafers)</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>~$100–$300/wafer (varies by test complexity)</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="inlineStr">
+        <is>
+          <t>Same (done in TW)</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>Wafer probe testing identifies good dies before packaging. Cost depends on number of test insertions, probe card costs (~$932/thousand probes), and test time. Test equipment ~8% of total fab equipment spend.</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>SemiconductorInsight (wafer test probe market); MDPI Electronics (multi-site test cost analysis)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="65" customHeight="1">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>Packaging – Standard (FC-BGA)</t>
+        </is>
+      </c>
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>Done in Taiwan; ~$8/unit</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>~$8/unit</t>
+        </is>
+      </c>
+      <c r="D43" s="12" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Flip-chip BGA is the standard package for most logic chips. Price is set by OSAT providers (ASE, SPIL, Amkor) and is location-independent since both use Taiwan OSAT.</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>Silicon Analysts 2026 (semiconductor cost guide); OSAT market data</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="65" customHeight="1">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>Packaging – InFO (Fan-Out WLP)</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>Done in Taiwan; ~$15/unit</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>~$15/unit</t>
+        </is>
+      </c>
+      <c r="D44" s="10" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>TSMC InFO used primarily for Apple A-series/M-series SoCs and MediaTek Dimensity. TSMC InFO revenue &gt;$3.5B/yr. Pricing identical since both sourced from TSMC Taiwan packaging.</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>Silicon Analysts 2026; SemiconductorX (InFO overview); TechTicker (FOWLP market)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="65" customHeight="1">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>Packaging – CoWoS-S (2.5D)</t>
+        </is>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>Done in Taiwan; ~$70/unit</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>~$70/unit</t>
+        </is>
+      </c>
+      <c r="D45" s="12" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>CoWoS-S is the dominant advanced package for AI/HPC chips (NVIDIA H100, AMD MI300). Demand exceeds supply by 40–50%, lead times 40–52 weeks. Prices rising ~20% over next 2 years.</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>Silicon Analysts 2026; smbom.com (TSMC price hikes); Morgan Stanley estimates</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="65" customHeight="1">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>Packaging – CoWoS-L (large interposer)</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>Done in Taiwan; ~$84–$98/unit (20–40% &gt; CoWoS-S)</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>~$84–$98/unit</t>
+        </is>
+      </c>
+      <c r="D46" s="10" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>CoWoS-L uses organic interposer for larger multi-die designs (NVIDIA B200 Blackwell). Higher cost due to interposer complexity and lower yields.</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>Silicon Analysts packaging calculator; NVIDIA B200 cost breakdown</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="65" customHeight="1">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>Packaging – SoIC (3D Stacking)</t>
+        </is>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>Done in Taiwan; ~$120/unit</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>~$120/unit</t>
+        </is>
+      </c>
+      <c r="D47" s="12" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>TSMC SoIC enables 3D die stacking for highest-density integration. Currently lowest-volume, highest-cost option. Pricing is TSMC-set and location-independent.</t>
+        </is>
+      </c>
+      <c r="F47" s="8" t="inlineStr">
+        <is>
+          <t>Silicon Analysts 2026; TSMC advanced packaging roadmap</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="65" customHeight="1">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>Full Backend Cost (H100-class AI chip)</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>~$750–$1,100/chip (CoWoS-S/L + test + dicing) + AZ freight</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>~$750–$1,100/chip (CoWoS-S/L + test + dicing)</t>
+        </is>
+      </c>
+      <c r="D48" s="10" t="inlineStr">
+        <is>
+          <t>AZ adds ~$50–$150 freight</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>NVIDIA H100 SXM5 total COGS ~$3,320; CoWoS-S packaging alone ~$750. NVIDIA B200 total COGS ~$6,400 with CoWoS-L ~$1,100. Backend is 20–30% of total chip cost for AI accelerators.</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>Silicon Analysts (H100/B200 cost breakdown); industry estimates</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="65" customHeight="1">
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>Backend as % of Total Chip Cost</t>
+        </is>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>~10–20% (standard); ~20–30% (AI/HPC with CoWoS)</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>~10–20% (standard); ~20–30% (AI/HPC with CoWoS)</t>
+        </is>
+      </c>
+      <c r="D49" s="12" t="inlineStr">
+        <is>
+          <t>Same % (same providers)</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Backend share is growing rapidly with advanced packaging complexity. OSAT providers raising prices 8–20%, memory packaging surcharges up 30%. Industry shift: backend becoming strategic differentiator.</t>
+        </is>
+      </c>
+      <c r="F49" s="8" t="inlineStr">
+        <is>
+          <t>SemiconductorX (backend overview); Silicon Analysts (chip price hikes 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="65" customHeight="1">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>OSAT Price Trend</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>8–20% price hikes (2025–2026)</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>8–20% price hikes (2025–2026)</t>
+        </is>
+      </c>
+      <c r="D50" s="10" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>ASE expects advanced packaging/testing revenue to double in 2026. Near 90% utilization driving pricing power. Memory packaging surcharges up 30% due to AI server demand.</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>Silicon Analysts (repricing wave); Digitimes Feb 2026 (ASE); SemiconductorX</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="25" customHeight="1">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>GROSS MARGIN COMPARISON</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n"/>
+      <c r="C51" s="5" t="n"/>
+      <c r="D51" s="5" t="n"/>
+      <c r="E51" s="5" t="n"/>
+      <c r="F51" s="5" t="n"/>
+    </row>
+    <row r="52" ht="65" customHeight="1">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>TSMC Corporate Gross Margin (2025)</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>59.9% full-year; 62.3% in Q4 2025</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>59.9% full-year; 62.3% in Q4 2025</t>
+        </is>
+      </c>
+      <c r="D52" s="10" t="inlineStr">
+        <is>
+          <t>N/A (consolidated)</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
+        <is>
+          <t>Company-wide margin. Up 3.8pp from 56.1% in 2024. Q4 2025 beat guidance (59–61%) by 1.3pp. Driven by N3 scaling, favorable FX, stronger pricing.</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>Finovian (TSMC Q4 2025 earnings); MacroTrends (TSM gross margin); TSMC Q4 2025 results</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="65" customHeight="1">
+      <c r="A53" s="8" t="inlineStr">
+        <is>
+          <t>TSMC Operating Margin (2025)</t>
+        </is>
+      </c>
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>50.8% full-year; 54.0% in Q4 2025</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>50.8% full-year; 54.0% in Q4 2025</t>
+        </is>
+      </c>
+      <c r="D53" s="12" t="inlineStr">
+        <is>
+          <t>N/A (consolidated)</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>Operating margin up 5.1pp from 45.7% in 2024. Net income ~$55.4B (NT$1,717B), +51.7% YoY.</t>
+        </is>
+      </c>
+      <c r="F53" s="8" t="inlineStr">
+        <is>
+          <t>Finovian (TSMC Q4 2025 earnings); TSMC investor relations</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="65" customHeight="1">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>Arizona Fab Estimated Gross Margin</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>~8% (5nm production, est. 2025)</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>~50–60% (mature Taiwan fabs)</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>AZ ~42–52pp lower</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
+        <is>
+          <t>AZ 5nm production estimated at ~8% gross margin per White Hsu / Taiwan Tech Dispatch analysis. Low margin reflects: (1) new fab depreciation, (2) ramp-up phase, (3) all hidden efficiencies priced explicitly in US system. This is expected to improve over time.</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="inlineStr">
+        <is>
+          <t>White Hsu Blog (TSMC AZ low margins, Feb 2026); mbi-deepdives.com (TSMC's Margins)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="65" customHeight="1">
+      <c r="A55" s="8" t="inlineStr">
+        <is>
+          <t>Arizona Fab Net Profit (2025)</t>
+        </is>
+      </c>
+      <c r="B55" s="8" t="inlineStr">
+        <is>
+          <t>NT$161.4B (~$5.15B) profit</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>N/A (not separately reported)</t>
+        </is>
+      </c>
+      <c r="D55" s="12" t="inlineStr">
+        <is>
+          <t>First profitable year</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>Dramatic turnaround from NT$142B loss in 2024 — a ~NT$300B swing. Driven by N4P ramp (began Q4 2024) + AI client demand. Government grants (25% of qualified investment) significantly aided financial performance.</t>
+        </is>
+      </c>
+      <c r="F55" s="8" t="inlineStr">
+        <is>
+          <t>BigGo Finance (TSMC AZ turnaround); TrendForce Mar 2026; AZ Tech Council; TSMC 2025 financial report</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="65" customHeight="1">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>Arizona Margin Dilution Impact</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>1–2% dilution to corporate margin (2025 est.)</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D56" s="10" t="inlineStr">
+        <is>
+          <t>Manageable</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
+        <is>
+          <t>Overseas fabs (AZ+Japan+Germany) expected to dilute corporate gross margin by 2–3% in early stages, widening to 3–4% at scale. 2025 revised down to 1–2%. TSMC mitigates with premium pricing for 'geographic flexibility.'</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>mbi-deepdives.com (TSMC's Margins); BeyondSPX (margin dilution analysis); Yahoo Finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="65" customHeight="1">
+      <c r="A57" s="8" t="inlineStr">
+        <is>
+          <t>Wafer Price Premium (AZ vs TW)</t>
+        </is>
+      </c>
+      <c r="B57" s="8" t="inlineStr">
+        <is>
+          <t>5–20% premium charged to customers</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>Baseline pricing</t>
+        </is>
+      </c>
+      <c r="D57" s="12" t="inlineStr">
+        <is>
+          <t>+5–20%</t>
+        </is>
+      </c>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>AMD CEO Lisa Su confirmed 5–20% premium for AZ-made chips. TSMC CEO C.C. Wei: charges for 'geographic flexibility' and considers 'made in USA' a premium product. Customers have agreed to pay premium.</t>
+        </is>
+      </c>
+      <c r="F57" s="8" t="inlineStr">
+        <is>
+          <t>The Verge (TSMC US chips premium); Yahoo Finance (TSMC AZ pricing); Taiwan News May 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="65" customHeight="1">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>Long-Term Margin Trajectory (AZ)</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>Improving toward ~30–40% (analyst consensus 3–5 yr)</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>Stable at ~50–60%</t>
+        </is>
+      </c>
+      <c r="D58" s="10" t="inlineStr">
+        <is>
+          <t>Gap narrowing over time</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
+        <is>
+          <t>AZ margins expected to improve as: (1) depreciation burden decreases, (2) yields improve (already 92% N4P vs 88% in Hsinchu), (3) local ecosystem matures, (4) Fab 2 &amp; 3 add scale. Unlikely to fully match Taiwan margins due to structural cost differences.</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="inlineStr">
+        <is>
+          <t>Digitimes (AZ profitability milestone); ainvest.com (TSMC AZ catalyst); analyst consensus</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="65" customHeight="1">
+      <c r="A59" s="8" t="inlineStr">
+        <is>
+          <t>Key Margin Differentiator</t>
+        </is>
+      </c>
+      <c r="B59" s="8" t="inlineStr">
+        <is>
+          <t>Cultural costs made explicit (formally priced labor, compliance, procedures)</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>Cultural efficiencies absorbed informally (unpaid OT, flexible roles, implicit response)</t>
+        </is>
+      </c>
+      <c r="D59" s="12" t="inlineStr">
+        <is>
+          <t>Structural</t>
+        </is>
+      </c>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>Per White Hsu analysis: Taiwan's high margins partly reflect 'invisible costs' — engineers returning to fabs without being called, blurred job roles, rapid cross-team action without formal escalation. In AZ, all these are formalized into explicit labor/compliance costs.</t>
+        </is>
+      </c>
+      <c r="F59" s="8" t="inlineStr">
+        <is>
+          <t>White Hsu Blog (TSMC AZ low margins, Feb 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="25" customHeight="1">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>OVERALL WAFER PROCESSING COST</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="n"/>
+      <c r="C60" s="5" t="n"/>
+      <c r="D60" s="5" t="n"/>
+      <c r="E60" s="5" t="n"/>
+      <c r="F60" s="5" t="n"/>
+    </row>
+    <row r="61" ht="65" customHeight="1">
+      <c r="A61" s="8" t="inlineStr">
+        <is>
+          <t>Total Wafer Processing Cost (300mm, N4/N3)</t>
+        </is>
+      </c>
+      <c r="B61" s="8" t="inlineStr">
+        <is>
+          <t>~$17,000–$22,000/wafer</t>
+        </is>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>~$15,500–$20,000/wafer</t>
+        </is>
+      </c>
+      <c r="D61" s="13" t="inlineStr">
+        <is>
+          <t>AZ ~10% higher overall</t>
+        </is>
+      </c>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>Per TechInsights Strategic Cost &amp; Price Model (Scotten Jones). Equipment dominance (~67%+ of cost) equalizes locations. Total difference is &lt;10%.</t>
+        </is>
+      </c>
+      <c r="F61" s="8" t="inlineStr">
+        <is>
+          <t>TechInsights Mar 2025 (Chip Insider, G. Dan Hutcheson); Silicon Analysts 2026; SemiWiki</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="65" customHeight="1">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>Total Chip Cost incl. Backend (AI/HPC)</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>~$3,500–$7,000/chip (wafer + backend + AZ freight)</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>~$3,300–$6,400/chip (wafer + backend)</t>
+        </is>
+      </c>
+      <c r="D62" s="11" t="inlineStr">
+        <is>
+          <t>AZ ~5–10% higher all-in</t>
+        </is>
+      </c>
+      <c r="E62" s="6" t="inlineStr">
+        <is>
+          <t>For AI accelerators (H100/B200 class). Frontend wafer cost is ~10% higher in AZ; backend costs identical (done in Taiwan); freight adds ~$50–150/wafer. All-in premium is lower than frontend-only premium.</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="inlineStr">
+        <is>
+          <t>Silicon Analysts (H100/B200 COGS); TechInsights; calculated</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="65" customHeight="1">
+      <c r="A63" s="8" t="inlineStr">
+        <is>
           <t>Operating Cost Premium (all-in)</t>
         </is>
       </c>
-      <c r="B40" s="6" t="inlineStr">
+      <c r="B63" s="8" t="inlineStr">
         <is>
           <t>Baseline + ~10%</t>
         </is>
       </c>
-      <c r="C40" s="6" t="inlineStr">
+      <c r="C63" s="8" t="inlineStr">
         <is>
           <t>Baseline</t>
         </is>
       </c>
-      <c r="D40" s="10" t="inlineStr">
+      <c r="D63" s="12" t="inlineStr">
         <is>
           <t>+10%</t>
         </is>
       </c>
-      <c r="E40" s="6" t="inlineStr">
+      <c r="E63" s="8" t="inlineStr">
         <is>
           <t>Final TechInsights assessment. Earlier estimates of 30–50%+ premiums were based on construction costs and flawed labor assumptions. Equipment parity is decisive.</t>
         </is>
       </c>
-      <c r="F40" s="6" t="inlineStr">
+      <c r="F63" s="8" t="inlineStr">
         <is>
           <t>TechInsights Mar 2025; TechPowerUp Feb 2025 &amp; Mar 2025; TechSpot Mar 2025</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="14">
     <mergeCell ref="A24:F24"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="A33:F33"/>
     <mergeCell ref="A38:F38"/>
     <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A51:F51"/>
+    <mergeCell ref="A60:F60"/>
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A5:F5"/>
@@ -1570,7 +2268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:D67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2443,6 +3141,446 @@
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>BigGo Finance – TSMC AZ $5.15B Profit Turnaround</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>https://finance.biggo.com/news/C_MZoZwBq7sy_YQMmt-O</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="8" t="n">
+        <v>44</v>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>TrendForce – TSMC 2025 Overseas Split</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>https://www.trendforce.com/news/2026/03/02/news-tsmcs-2025-overseas-split-china-leads-profits-arizona-turns-profitable-japan-losses-triple/</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>White Hsu Blog – TSMC AZ Fab Low Margins</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>https://whitehsu.blog/2026/02/09/tsmc-arizona-fab-low-margins/</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>Feb 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="8" t="n">
+        <v>46</v>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>Finovian – TSMC Q4 2025 Earnings (62.3% GM)</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>https://finovian.com/category/earnings/tsmc-q4-2025-earnings-explained/</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Q4 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>mbi-deepdives.com – TSMC's Margins</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>https://www.mbi-deepdives.com/tsmcs-margins/</t>
+        </is>
+      </c>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="8" t="n">
+        <v>48</v>
+      </c>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>BeyondSPX – TSMC AI Supremacy &amp; Margin Dilution</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>https://beyondspx.com/quote/TSM/tsmc-s-ai-supremacy-meets-global-reality-why-margin-dilution-is-a-feature-not-a-bug-nyse-tsm</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="6" t="n">
+        <v>49</v>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>The Verge – TSMC US Chips Price Premium</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>https://on.theverge.com/news/712904/tsmcs-us-chips-come-at-a-premium</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>Taiwan News – TSMC 30% Price Hike AZ Chips</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>https://www.taiwannews.com.tw/news/6114167</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>May 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="6" t="n">
+        <v>51</v>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>Yahoo Finance – TSMC AZ Fab 21 Higher Price</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/news/tsmcs-arizona-fab-21-mass-114824172.html</t>
+        </is>
+      </c>
+      <c r="D54" s="6" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="22" customHeight="1">
+      <c r="A55" s="8" t="n">
+        <v>52</v>
+      </c>
+      <c r="B55" s="8" t="inlineStr">
+        <is>
+          <t>Silicon Analysts – Semiconductor Cost Guide 2026</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>https://siliconanalysts.com/guide/semiconductor-costs</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="6" t="n">
+        <v>53</v>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>Silicon Analysts – Chip Price Hikes 2026</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>https://siliconanalysts.com/analysis/semiconductor-repricing-wave-price-hikes-reshape-chip-supply-chain</t>
+        </is>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="22" customHeight="1">
+      <c r="A57" s="8" t="n">
+        <v>54</v>
+      </c>
+      <c r="B57" s="8" t="inlineStr">
+        <is>
+          <t>Silicon Analysts – NVIDIA B200 Cost Breakdown</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>https://siliconanalysts.com/analysis/nvidia-b200-blackwell-cost-breakdown</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="22" customHeight="1">
+      <c r="A58" s="6" t="n">
+        <v>55</v>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>Silicon Analysts – Adv. Packaging Cost Calculator</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>https://siliconanalysts.com/tools/packaging</t>
+        </is>
+      </c>
+      <c r="D58" s="6" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="22" customHeight="1">
+      <c r="A59" s="8" t="n">
+        <v>56</v>
+      </c>
+      <c r="B59" s="8" t="inlineStr">
+        <is>
+          <t>SemiconductorX – Backend Assembly &amp; Test Overview</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>https://www.semiconductorx.com/back-end-assembly-overview.html</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="22" customHeight="1">
+      <c r="A60" s="6" t="n">
+        <v>57</v>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>SemiWiki – TSMC AZ Chips Flown to Taiwan</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>https://semiwiki.com/forum/threads/tsmc-arizona-chips-are-reportedly-being-flown-back-to-taiwan-for-packaging-u-s-semiconductor-supply-chain-still-remains-dependent-on-taiwan.23109/</t>
+        </is>
+      </c>
+      <c r="D60" s="6" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="22" customHeight="1">
+      <c r="A61" s="8" t="n">
+        <v>58</v>
+      </c>
+      <c r="B61" s="8" t="inlineStr">
+        <is>
+          <t>Digitimes – TSMC AZ Profitability Milestone</t>
+        </is>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>https://www.digitimes.com/news/a20260302VL210/tsmc-arizona-fab-profit-2025.html</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="22" customHeight="1">
+      <c r="A62" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>Digitimes – ASE Advanced Packaging Revenue 2x</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>https://www.digitimes.com/news/a20260206PD224/packaging-ase-2026-testing-osat.html</t>
+        </is>
+      </c>
+      <c r="D62" s="6" t="inlineStr">
+        <is>
+          <t>Feb 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="22" customHeight="1">
+      <c r="A63" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="B63" s="8" t="inlineStr">
+        <is>
+          <t>AZ Tech Council – TSMC AZ First Profit</t>
+        </is>
+      </c>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>https://www.aztechcouncil.org/tsmcs-arizona-fab-generates-first-profit/</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="22" customHeight="1">
+      <c r="A64" s="6" t="n">
+        <v>61</v>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>Astute Analytica – Wafer Dicing Services Market</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr">
+        <is>
+          <t>https://www.astuteanalytica.com/industry-report/wafer-dicing-services-market</t>
+        </is>
+      </c>
+      <c r="D64" s="6" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="22" customHeight="1">
+      <c r="A65" s="8" t="n">
+        <v>62</v>
+      </c>
+      <c r="B65" s="8" t="inlineStr">
+        <is>
+          <t>MacroTrends – TSMC Gross Margin History</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>https://www.macrotrends.net/stocks/charts/TSM/taiwan-semiconductor-manufacturing/gross-margin</t>
+        </is>
+      </c>
+      <c r="D65" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="22" customHeight="1">
+      <c r="A66" s="6" t="n">
+        <v>63</v>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>ainvest.com – TSMC AZ Bet Valuation Analysis</t>
+        </is>
+      </c>
+      <c r="C66" s="6" t="inlineStr">
+        <is>
+          <t>https://www.ainvest.com/news/tsmc-arizona-bet-catalyst-valuation-costly-distraction-2601/</t>
+        </is>
+      </c>
+      <c r="D66" s="6" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="22" customHeight="1">
+      <c r="A67" s="8" t="n">
+        <v>64</v>
+      </c>
+      <c r="B67" s="8" t="inlineStr">
+        <is>
+          <t>Wafer World – Guide to Wafer Shipping</t>
+        </is>
+      </c>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>https://www.waferworld.com/post/guide-to-wafer-shipping</t>
+        </is>
+      </c>
+      <c r="D67" s="8" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
@@ -2463,7 +3601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2577,6 +3715,56 @@
         </is>
       </c>
     </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>GROSS MARGIN: Arizona fab estimated at ~8% gross margin (5nm) vs ~50–60% for mature Taiwan fabs. The gap reflects new-fab depreciation, ramp-up costs, and explicit pricing of cultural efficiencies that are absorbed informally in Taiwan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>GROSS MARGIN: TSMC Arizona posted NT$161.4B ($5.15B) profit in 2025 — a dramatic turnaround from NT$142B loss in 2024. Government grants (25% of qualified investment) were critical. Corporate gross margin: 59.9% (2025), 62.3% in Q4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="45" customHeight="1">
+      <c r="A15" s="14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="15" t="inlineStr">
+        <is>
+          <t>GROSS MARGIN: TSMC charges a 5–20% wafer price premium for Arizona-made chips (per AMD CEO Lisa Su). CEO C.C. Wei frames it as charging for 'geographic flexibility' and 'made in USA' premium.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>BACKEND COSTS: All Arizona wafers currently ship back to Taiwan for dicing, testing, and packaging — adding ~$50–$150/wafer in air freight but using the same OSAT infrastructure as Taiwan-made wafers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>BACKEND COSTS: Advanced packaging (CoWoS-S at ~$70/unit, CoWoS-L at ~$84–98/unit, SoIC at ~$120/unit) is identical in cost for AZ and TW wafers since all packaging is done in Taiwan. Backend is 10–20% of standard chip cost, rising to 20–30% for AI/HPC with CoWoS.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>

</xml_diff>